<commit_message>
Strip revision narration from Draft_016 and Excel; corrections only
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="B2:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -645,11 +645,10 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Compiled Hedging Codings — PSAU Corpus (Draft_002 / Thesis Draft_016)</t>
+          <t>Compiled Hedging Codings — PSAU Corpus</t>
         </is>
       </c>
     </row>
@@ -660,7 +659,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -2683,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="B2:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2698,7 +2696,6 @@
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="17" t="inlineStr">
         <is>
@@ -2706,7 +2703,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -5373,7 +5369,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible. Recoded from FP-Gen in Draft_016.</t>
+          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible.</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5412,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'their quorum quenching activities' asserts the activities exist. Recoded from FP-Gen in Draft_016.</t>
+          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'their quorum quenching activities' asserts the activities exist.</t>
         </is>
       </c>
     </row>
@@ -5459,7 +5455,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'public health concerns' asserted as fact vs possible. Same abstract retains conclusion-position 'potential public health risks' as EC; consistent under Working Test. Recoded from FP-Gen in Draft_016.</t>
+          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'public health concerns' asserted as fact vs possible. Same abstract also codes conclusion-position 'potential public health risks' as EC.</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5498,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'posed health risks' asserts risks as fact. Recoded from FP-Gen in Draft_016.</t>
+          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'posed health risks' asserts risks as fact.</t>
         </is>
       </c>
     </row>
@@ -5545,7 +5541,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens. Recoded from FP-Gen in Draft_016.</t>
+          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="B2:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5573,7 +5569,6 @@
     <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="17" t="inlineStr">
         <is>
@@ -5581,7 +5576,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -6925,7 +6919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="B2:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6938,7 +6932,6 @@
     <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="17" t="inlineStr">
         <is>
@@ -6946,7 +6939,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -9030,7 +9022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="B2:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9043,7 +9035,6 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="17" t="inlineStr">
         <is>
@@ -9054,11 +9045,10 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Final coded output for the 60-abstract PSAU corpus, coded per the Hedging Codebook (Draft_016 Working Test recode of 5 borderline potential tokens).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Final coded output for the 60-abstract PSAU corpus, coded per the Hedging Codebook.</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Strip all revision narration from Draft_016 and Excel; present-tense decision rules only
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H101"/>
+  <dimension ref="B1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -645,6 +645,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -659,6 +660,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -803,6 +805,8 @@
         <v>0.47</v>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -896,6 +900,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -995,6 +1001,8 @@
         <v>38</v>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -1064,13 +1072,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>Source: 005_CorpusCoverted.docx (60 abstracts). Coded per Hedging Codebook (rebuilt, with user's manual corrections folded in). All decisions in 'Hedges', 'Unhedged Sites', and 'Rejected Candidates' sheets.</t>
-        </is>
-      </c>
-    </row>
+          <t>Source: 005_CorpusCoverted.docx (60 abstracts). Coded per Hedging Codebook. All decisions in 'Hedges', 'Unhedged Sites', and 'Rejected Candidates' sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -2789,7 +2801,7 @@
       </c>
       <c r="J5" s="21" t="inlineStr">
         <is>
-          <t>Lexical hedge: 'implies' functions as 'suggest' (extensions note).</t>
+          <t>Lexical hedge: 'implies' functions as 'suggest'.</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3446,7 @@
       </c>
       <c r="J20" s="23" t="inlineStr">
         <is>
-          <t>Adverbial hedge: 'potentially' qualifies the claim (extensions note).</t>
+          <t>Adverbial hedge: 'potentially' qualifies the claim.</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4693,7 @@
       </c>
       <c r="J49" s="21" t="inlineStr">
         <is>
-          <t>Modal hedge: 'it can be derived that the application of different alternative rooting hormones has a comparable effect' — inferential hedge per extensions note.</t>
+          <t>Modal hedge: 'it can be derived that the application of different alternative rooting hormones has a comparable effect'.</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4865,7 @@
       </c>
       <c r="J53" s="21" t="inlineStr">
         <is>
-          <t>Modal hedge: 'can be attributed to the nutrient-rich content' — inferential hedge per extensions note.</t>
+          <t>Modal hedge: 'can be attributed to the nutrient-rich content'.</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5037,7 @@
       </c>
       <c r="J57" s="21" t="inlineStr">
         <is>
-          <t>Modal hedge: 'It can also be concluded that D1 rice bran mixed with water spinach... can help minimize the cost of production' — inferential hedge per extensions note.</t>
+          <t>Modal hedge: 'It can also be concluded that D1 rice bran mixed with water spinach... can help minimize the cost of production'.</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5123,7 @@
       </c>
       <c r="J59" s="21" t="inlineStr">
         <is>
-          <t>Modal hedge: 'insect farming can be seen as a potential solution' — inferential hedge per extensions note.</t>
+          <t>Modal hedge: 'insect farming can be seen as a potential solution'.</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5295,7 @@
       </c>
       <c r="J63" s="21" t="inlineStr">
         <is>
-          <t>Modal hedge: 'it can be stated that the ratio of 70% guinea grass (GG) + 30% concentrate (C)... had a significantly higher feed conversion ratio' — inferential hedge per extensions note.</t>
+          <t>Modal hedge: 'it can be stated that the ratio of 70% guinea grass (GG) + 30% concentrate (C)... had a significantly higher feed conversion ratio'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Draft_017: align prose with tables/Excel after recodes
- Fix stale counts (65 hedges, 41 lexical, 32 unhedged-in-zero, FP 32/14, density lead 0.01)
- Extensions: topic-naming (FP-Gen); remove orange color spill
- Pro forma definition aligned to Part IV wording
- Sensitivity paragraph for potential / KW
- Working Test override example (B11) added to decision rules
- Soften booster absolute pending recount on 25
- Excel Summary Layer 1 percentages corrected
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -848,7 +848,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>35.0%</t>
+          <t>32.3%</t>
         </is>
       </c>
     </row>
@@ -860,11 +860,11 @@
       </c>
       <c r="C16" s="11" t="inlineStr"/>
       <c r="D16" s="9" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>63.1%</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.6%</t>
         </is>
       </c>
     </row>
@@ -1072,8 +1072,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36"/>
     <row r="37">
       <c r="B37" s="16" t="inlineStr">
         <is>
@@ -1081,8 +1079,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="B40" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel: strip residual revision phrasing; mark ambiguous cases [AMB]
- "Per revised rule" → "Per Decision Rules"
- [AMB] on Working Test hedges (B11, B12, B16, VM9, Aas5) and borderline FPs
- Thesis already free of revision narration; clarifications retained
- References complete vs Draft 7 (+ Landis for kappa)
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="B2:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -645,7 +645,6 @@
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -660,7 +659,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -805,8 +803,6 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -900,8 +896,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1001,8 +995,6 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -2689,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J69"/>
+  <dimension ref="A2:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5377,7 +5369,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'presence of mycobacterial infections' asserts existence; 'potential mycobacterial infections' marks them as possible.</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5412,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'their quorum quenching activities' asserts the activities exist.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'their quorum quenching activities' asserts the activities exist.</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5455,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'public health concerns' asserted as fact vs possible. Same abstract also codes conclusion-position 'potential public health risks' as EC.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'public health concerns' asserted as fact vs possible. Same abstract also codes conclusion-position 'potential public health risks' as EC.</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5498,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'posed health risks' asserts risks as fact.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'posed health risks' asserts risks as fact.</t>
         </is>
       </c>
     </row>
@@ -5549,7 +5541,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Lexical hedge (Working Test): removing 'potential' changes commitment — 'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
+          <t>[AMB] Lexical hedge (Working Test): removing 'potential' changes commitment — 'a solution' is stronger endorsement than 'a potential solution'. Multi-hedge isolation: 'can' already coded EC in same sentence; 'potential' independently softens.</t>
         </is>
       </c>
     </row>
@@ -6927,7 +6919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H62"/>
+  <dimension ref="A2:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7050,7 +7042,7 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>Factive reporting: 'Results indicated that... exhibited a notable increase' — synonym for 'showed', reports results as settled fact. Per Decision Rules: not a hedge when used as synonym for showed/demonstrated.</t>
+          <t>[AMB] Factive reporting: 'Results indicated that... exhibited a notable increase' — synonym for 'showed', reports results as settled fact. Per Decision Rules: not a hedge when used as synonym for showed/demonstrated.</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7742,7 @@
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>Factive reporting: 'significant differences in melting temperature indicate variations in thermal stability' — direct logical entailment from statistical significance, not a hedged inference. Per Decision Rules: synonym for showed/demonstrated.</t>
+          <t>[AMB] Factive reporting: 'significant differences in melting temperature indicate variations in thermal stability' — direct logical entailment from statistical significance, not a hedged inference. Per Decision Rules: synonym for showed/demonstrated.</t>
         </is>
       </c>
     </row>
@@ -8100,7 +8092,7 @@
       </c>
       <c r="H36" s="21" t="inlineStr">
         <is>
-          <t>Factive reporting: 'The results indicate that the mean effect... varied' — factive reporting of a statistical outcome, synonym for 'showed'. Per Decision Rules: not a hedge when used as synonym for showed/demonstrated.</t>
+          <t>[AMB] Factive reporting: 'The results indicate that the mean effect... varied' — factive reporting of a statistical outcome, synonym for 'showed'. Per Decision Rules: not a hedge when used as synonym for showed/demonstrated.</t>
         </is>
       </c>
     </row>
@@ -8415,7 +8407,7 @@
       </c>
       <c r="H45" s="21" t="inlineStr">
         <is>
-          <t>Factive reporting: 'Multiple regression analysis indicated that knowledge significantly predicted self-assessed awareness' — factive reporting of regression output, synonym for 'showed'. Per Decision Rules: not a hedge when used as synonym for showed/demonstrated.</t>
+          <t>[AMB] Factive reporting: 'Multiple regression analysis indicated that knowledge significantly predicted self-assessed awareness' — factive reporting of regression output, synonym for 'showed'. Per Decision Rules: not a hedge when used as synonym for showed/demonstrated.</t>
         </is>
       </c>
     </row>
@@ -8555,7 +8547,7 @@
       </c>
       <c r="H49" s="21" t="inlineStr">
         <is>
-          <t>Capability: 'can significantly enhance' — can + active content verb (enhance) describing a treatment effect. Per revised rule: can + enhance/promote/reduce/help = capability regardless of clause embedding. Working Test: remove 'can' alone, 'suggests that... significantly enhances' remains fully hedged by 'suggests.'.</t>
+          <t>[AMB] Capability: 'can significantly enhance' — can + active content verb (enhance) describing a treatment effect. Per Decision Rules: can + enhance/promote/reduce/help = capability regardless of clause embedding. Working Test: remove 'can' alone, 'suggests that... significantly enhances' remains fully hedged by 'suggests.'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: separate P/DO/REC function coding sheet; [AMB] markers
- New sheet 'P and DO Functions': DO connectors and REC prescriptions coded
  regardless of hedge status; P absent in corpus
- [AMB] on Working Test and borderline Decision-Rules cases
- No classic politeness formulas found in abstracts
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unhedged Sites" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected Candidates" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P and DO Functions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,6 +108,9 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="10">
@@ -201,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -267,6 +271,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2681,7 +2686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J69"/>
+  <dimension ref="B2:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -6919,7 +6924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H62"/>
+  <dimension ref="B2:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9539,4 +9544,1068 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>Abstract ID</t>
+        </is>
+      </c>
+      <c r="B1" s="37" t="inlineStr">
+        <is>
+          <t>Discipline</t>
+        </is>
+      </c>
+      <c r="C1" s="37" t="inlineStr">
+        <is>
+          <t>Phrase / Token</t>
+        </is>
+      </c>
+      <c r="D1" s="37" t="inlineStr">
+        <is>
+          <t>Context (short)</t>
+        </is>
+      </c>
+      <c r="E1" s="37" t="inlineStr">
+        <is>
+          <t>Function Code</t>
+        </is>
+      </c>
+      <c r="F1" s="37" t="inlineStr">
+        <is>
+          <t>Hedge Status</t>
+        </is>
+      </c>
+      <c r="G1" s="37" t="inlineStr">
+        <is>
+          <t>Ambiguous</t>
+        </is>
+      </c>
+      <c r="H1" s="37" t="inlineStr">
+        <is>
+          <t>Reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Thus</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Thus, in the optimization process...</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Discourse connector sequencing problem to method.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hence / thus</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hence, biosynthesis is feasible; thus making a remarkable choice</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Claim-sequence connectors; hedge if any is separate (may).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Thus</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Thus, the researcher provided a policy proposal...</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Results-to-recommendation connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hence</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Hence, this study aimed to investigate...</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Background-to-aim connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hence</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Hence, LAB have emerged as a focal point...</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Problem-to-focus connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B16</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Thus</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Thus, this study detected the presence...</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Rationale-to-aim connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hence / Thus</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Hence / Thus linking to recommendations</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Problem/findings to recommendation moves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Hence</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hence, the study aimed to investigate...</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Background-to-aim connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VM7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Thus</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Thus, no significant association could be established</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Results-to-conclusion connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>VM9</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>hence</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>hence, all individual shrimps counted as one sample</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Methods sequencing only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>VM12</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hence</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hence, this study aimed to detect ASF virus...</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Not a hedge</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Background-to-aim connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Further studies are recommended to confirm...</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Further-research prescription; deontic, not politeness (P).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>should</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>proper waste management should be established</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Deontic prescription; not face-softening (P).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>should</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Further studies should focus on isolation...</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Further-research recommendation move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>B19</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>should</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>approaches should be considered; government should address</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Deontic recommendations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>VM7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>needed</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Further research is needed to validate</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Further-research recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>VM9</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>recommend</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>findings recommend removing the shrimp's GIT</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Deontic prescription from findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>VM12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>it is recommended to consider monitoring...</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Deontic recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>VM20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Veterinary Medicine</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>stricter guidelines are recommended</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Deontic policy recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Acs8</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>recommends</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>The researcher recommends foliar and drenching...</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Author recommendation move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Aas8</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>it is recommended to feed mallard ducks...</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Deontic recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Aas9</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>it is recommended for future researchers...</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Further-research recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Aas10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>researchers still recommended incorporating...</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FP-Rec</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Deontic recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>All disciplines</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>(no classic P formulas)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>No as-X-suggested / in-our-view / please / kindly / it-should-be-noted</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Absent in corpus</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>No politeness-deference hedges attested in these abstracts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: Layer 2 is only EC/P/DO; FP-Rec is a reject reason, not a function
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -9552,7 +9552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9578,12 +9578,12 @@
       </c>
       <c r="E1" s="37" t="inlineStr">
         <is>
-          <t>Function Code</t>
+          <t>Function Code (EC/P/DO only)</t>
         </is>
       </c>
       <c r="F1" s="37" t="inlineStr">
         <is>
-          <t>Hedge Status</t>
+          <t>Hedge? (Y/N)</t>
         </is>
       </c>
       <c r="G1" s="37" t="inlineStr">
@@ -9625,7 +9625,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Discourse connector sequencing problem to method.</t>
+          <t>Discourse connector sequencing problem to method; organizes research moves, not epistemic hedge.</t>
         </is>
       </c>
     </row>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -9677,7 +9677,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Claim-sequence connectors; hedge if any is separate (may).</t>
+          <t>Claim-sequence connectors; any hedge is separate (may).</t>
         </is>
       </c>
     </row>
@@ -9709,7 +9709,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -9751,7 +9751,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -9793,7 +9793,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hence / Thus linking to recommendations</t>
+          <t>Hence / Thus linking problem/findings to recommendations</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -9877,7 +9877,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -9961,7 +9961,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -10045,7 +10045,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Not a hedge</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -10062,546 +10062,84 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>All disciplines</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>recommended</t>
+          <t>(no classic P formulas)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Further studies are recommended to confirm...</t>
+          <t>No "as X suggested", "in our view", "please", "kindly", "it should be noted"</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>REC</t>
+          <t>P</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FP-Rec</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Further-research prescription; deontic, not politeness (P).</t>
+          <t>No politeness-deference devices attested. Layer 2 P = 0 in this corpus.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>NOTE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>should</t>
+          <t>should / recommended / needed</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>proper waste management should be established</t>
+          <t>See Rejected Candidates (FP-Rec)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>REC</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FP-Rec</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Deontic prescription; not face-softening (P).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>B17</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>should</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Further studies should focus on isolation...</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Further-research recommendation move.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>B19</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>should</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>approaches should be considered; government should address</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Deontic recommendations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>VM7</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>needed</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Further research is needed to validate</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Further-research recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>VM9</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>recommend</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>findings recommend removing the shrimp's GIT</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Deontic prescription from findings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>VM12</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>it is recommended to consider monitoring...</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Deontic recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>VM20</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Veterinary Medicine</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>stricter guidelines are recommended</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Deontic policy recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Acs8</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>recommends</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>The researcher recommends foliar and drenching...</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Author recommendation move.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Aas8</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>it is recommended to feed mallard ducks...</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Deontic recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Aas9</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>it is recommended for future researchers...</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Further-research recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Aas10</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>researchers still recommended incorporating...</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>REC</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>FP-Rec</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Deontic recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>All disciplines</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>(no classic P formulas)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>No as-X-suggested / in-our-view / please / kindly / it-should-be-noted</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Absent in corpus</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>No politeness-deference hedges attested in these abstracts.</t>
+          <t>FP-Rec is a false-positive REASON CODE (deontic prescription), not a Layer 2 function. Layer 2 is only EC, P, DO. These remain rejected as non-hedges.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Second pass: tag remaining DO (Therefore, In conclusion); P still absent
</commit_message>
<xml_diff>
--- a/thesis/007_CompiledResult_Draft_002.xlsx
+++ b/thesis/007_CompiledResult_Draft_002.xlsx
@@ -9552,7 +9552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9578,7 +9578,7 @@
       </c>
       <c r="E1" s="37" t="inlineStr">
         <is>
-          <t>Function Code (EC/P/DO only)</t>
+          <t>Function (EC/P/DO)</t>
         </is>
       </c>
       <c r="F1" s="37" t="inlineStr">
@@ -9610,12 +9610,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Thus</t>
+          <t>Thus / Therefore</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Thus, in the optimization process...</t>
+          <t>Thus, in the optimization process...; Therefore, further research will...</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Discourse connector sequencing problem to method; organizes research moves, not epistemic hedge.</t>
+          <t>Move connectors (problem→method; limit→future work). Not epistemic hedges.</t>
         </is>
       </c>
     </row>
@@ -9657,7 +9657,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hence, biosynthesis is feasible; thus making a remarkable choice</t>
+          <t>Hence, the biosynthesis is feasible; thus making a remarkable choice; thus demonstrating...</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -9677,7 +9677,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Claim-sequence connectors; any hedge is separate (may).</t>
+          <t>Claim-sequence connectors. Hedge if any is separate (may).</t>
         </is>
       </c>
     </row>
@@ -9719,7 +9719,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Results-to-recommendation connector.</t>
+          <t>Results→recommendation connector.</t>
         </is>
       </c>
     </row>
@@ -9761,7 +9761,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Background-to-aim connector.</t>
+          <t>Background→aim connector.</t>
         </is>
       </c>
     </row>
@@ -9803,7 +9803,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Problem-to-focus connector.</t>
+          <t>Problem→focus connector.</t>
         </is>
       </c>
     </row>
@@ -9820,12 +9820,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Thus</t>
+          <t>Thus / therefore</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Thus, this study detected the presence...</t>
+          <t>Thus, this study detected...; This study, therefore, underscores...</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -9845,7 +9845,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Rationale-to-aim connector.</t>
+          <t>Rationale→aim / findings→implication connectors.</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hence / Thus linking problem/findings to recommendations</t>
+          <t>Hence, sustainable planning should...; Thus, local government should...</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Problem/findings to recommendation moves.</t>
+          <t>Problem/findings→recommendation connectors.</t>
         </is>
       </c>
     </row>
@@ -9904,12 +9904,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hence</t>
+          <t>Therefore / Hence</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hence, the study aimed to investigate...</t>
+          <t>Therefore, this study aims...; Hence, the study aimed...</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -9929,7 +9929,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Background-to-aim connector.</t>
+          <t>Background→aim connectors.</t>
         </is>
       </c>
     </row>
@@ -9971,7 +9971,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Results-to-conclusion connector.</t>
+          <t>Results→conclusion connector.</t>
         </is>
       </c>
     </row>
@@ -10055,34 +10055,34 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Background-to-aim connector.</t>
+          <t>Background→aim connector.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Acs5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>All disciplines</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>(no classic P formulas)</t>
+          <t>Therefore</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>No "as X suggested", "in our view", "please", "kindly", "it should be noted"</t>
+          <t>Therefore, the... (yield inference connector)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -10092,54 +10092,390 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>No politeness-deference devices attested. Layer 2 P = 0 in this corpus.</t>
+          <t>Results→inference connector.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Aas9</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Therefore</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Therefore, it is recommended for future researchers...</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Results→recommendation connector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Acs3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>In conclusion</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>In conclusion, the number of rooted...</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Meta-textual framing of conclusion move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Acs7</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>In conclusion</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>In conclusion, the use of rice hull...</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Meta-textual framing of conclusion move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Acs10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>In conclusion</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>In conclusion, T3:...</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Meta-textual framing of conclusion move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Aas3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>In conclusion</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>In conclusion, proved the treatment 1...</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Meta-textual framing of conclusion move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Aas10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>In conclusion</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>In conclusion, based on the results, it can be stated...</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Meta-textual framing of conclusion move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>All disciplines</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>No "as X suggested", "in our view", "please", "kindly", "with due respect", "one might argue"</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>No politeness/deference devices in the 60 abstracts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>should / recommended / needed</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>See Rejected Candidates (FP-Rec)</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>regarding / with regard to / overall / first-second</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Common in VM KAP and ranking sentences</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>FP-Rec is a false-positive REASON CODE (deontic prescription), not a Layer 2 function. Layer 2 is only EC, P, DO. These remain rejected as non-hedges.</t>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Topic prepositions and ordinal ranking of results are NOT discourse-organization function. Left untagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>should / recommended (FP-Rec)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>See Rejected Candidates</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Deontic prescriptions. Reject reason FP-Rec, not Layer 2 P or DO.</t>
         </is>
       </c>
     </row>

</xml_diff>